<commit_message>
Agrega cantidad de preguntas, descripcion de competencias y meta institucional al dashboard
Muestra el numero de preguntas por TA1/TA2 (global y por carrera), agrega
tooltips con la descripcion oficial de cada competencia (extraida de
Cuadros_oficiales_por_carrera.xlsx) y suma una columna Meta >=70% en el
mapa de calor que marca si cada competencia cumple la meta institucional
de Satisfactorio + Sobresaliente.
</commit_message>
<xml_diff>
--- a/data/Cuadros_oficiales_por_carrera.xlsx
+++ b/data/Cuadros_oficiales_por_carrera.xlsx
@@ -106,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,6 +154,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -519,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I71"/>
+  <dimension ref="A1:J71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -528,6 +532,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -544,20 +549,13 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>══ TA1 — 240 estudiantes ══</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -565,14 +563,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -686,20 +676,13 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -747,6 +730,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -782,6 +770,11 @@
       <c r="I12" s="8" t="n">
         <v>20.8</v>
       </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>Diseña proyectos empresariales mediante análisis cuantitativo y metodologías de gestión, modelando escenarios organizacionales y asignando recursos, con rigor técnico, cumplimiento de objetivos y eficiencia operativa.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -817,6 +810,11 @@
       <c r="I13" s="12" t="n">
         <v>5.8</v>
       </c>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>Analiza mercados y entornos competitivos para estructurar estrategias de posicionamiento empresarial, utilizando segmentación y estudios de demanda, con diferenciación estratégica y generación de ventaja competitiva medible.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -852,6 +850,11 @@
       <c r="I14" s="8" t="n">
         <v>20</v>
       </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>Evalúa alternativas financieras y estructuras de inversión en organizaciones productivas o de servicios, aplicando herramientas de análisis económico y proyecciones financieras, con sustento cuantitativo, precisión técnica y control del riesgo.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -887,6 +890,11 @@
       <c r="I15" s="12" t="n">
         <v>21.2</v>
       </c>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>Formula estrategias y modelos de desarrollo empresarial en organizaciones públicas o privadas, con coherencia sistémica, visión directiva, capacidad de liderazgo estratégico y orientación a resultados verificables.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -922,6 +930,11 @@
       <c r="I16" s="8" t="n">
         <v>20.8</v>
       </c>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -957,6 +970,11 @@
       <c r="I17" s="12" t="n">
         <v>5.8</v>
       </c>
+      <c r="J17" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -992,6 +1010,11 @@
       <c r="I18" s="8" t="n">
         <v>20</v>
       </c>
+      <c r="J18" s="22" t="inlineStr">
+        <is>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -1027,21 +1050,19 @@
       <c r="I19" s="12" t="n">
         <v>21.2</v>
       </c>
-    </row>
+      <c r="J19" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="6" t="n"/>
-      <c r="I21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -1086,12 +1107,6 @@
           <t>CE2 / CT2</t>
         </is>
       </c>
-      <c r="C24" s="16" t="n"/>
-      <c r="D24" s="16" t="n"/>
-      <c r="E24" s="16" t="n"/>
-      <c r="F24" s="16" t="n"/>
-      <c r="G24" s="16" t="n"/>
-      <c r="H24" s="16" t="n"/>
       <c r="I24" s="17" t="n">
         <v>38.3</v>
       </c>
@@ -1122,30 +1137,18 @@
           <t>CE4 / CT4</t>
         </is>
       </c>
-      <c r="C26" s="16" t="n"/>
-      <c r="D26" s="16" t="n"/>
-      <c r="E26" s="16" t="n"/>
-      <c r="F26" s="16" t="n"/>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="16" t="n"/>
       <c r="I26" s="17" t="n">
         <v>46.7</v>
       </c>
     </row>
+    <row r="27"/>
+    <row r="28"/>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B29" s="6" t="n"/>
-      <c r="C29" s="6" t="n"/>
-      <c r="D29" s="6" t="n"/>
-      <c r="E29" s="6" t="n"/>
-      <c r="F29" s="6" t="n"/>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
-      <c r="I29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1190,12 +1193,6 @@
           <t>CE4 / CT4</t>
         </is>
       </c>
-      <c r="C32" s="16" t="n"/>
-      <c r="D32" s="16" t="n"/>
-      <c r="E32" s="16" t="n"/>
-      <c r="F32" s="16" t="n"/>
-      <c r="G32" s="16" t="n"/>
-      <c r="H32" s="16" t="n"/>
       <c r="I32" s="19" t="n">
         <v>95</v>
       </c>
@@ -1215,20 +1212,14 @@
         <v>91.2</v>
       </c>
     </row>
+    <row r="34"/>
+    <row r="35"/>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
           <t>══ TA2 — 63 estudiantes ══</t>
         </is>
       </c>
-      <c r="B36" s="4" t="n"/>
-      <c r="C36" s="4" t="n"/>
-      <c r="D36" s="4" t="n"/>
-      <c r="E36" s="4" t="n"/>
-      <c r="F36" s="4" t="n"/>
-      <c r="G36" s="4" t="n"/>
-      <c r="H36" s="4" t="n"/>
-      <c r="I36" s="4" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
@@ -1236,14 +1227,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B37" s="6" t="n"/>
-      <c r="C37" s="6" t="n"/>
-      <c r="D37" s="6" t="n"/>
-      <c r="E37" s="6" t="n"/>
-      <c r="F37" s="6" t="n"/>
-      <c r="G37" s="6" t="n"/>
-      <c r="H37" s="6" t="n"/>
-      <c r="I37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
@@ -1357,20 +1340,13 @@
         </is>
       </c>
     </row>
+    <row r="41"/>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B42" s="6" t="n"/>
-      <c r="C42" s="6" t="n"/>
-      <c r="D42" s="6" t="n"/>
-      <c r="E42" s="6" t="n"/>
-      <c r="F42" s="6" t="n"/>
-      <c r="G42" s="6" t="n"/>
-      <c r="H42" s="6" t="n"/>
-      <c r="I42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
@@ -1418,6 +1394,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J43" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
@@ -1453,6 +1434,11 @@
       <c r="I44" s="8" t="n">
         <v>3.2</v>
       </c>
+      <c r="J44" s="22" t="inlineStr">
+        <is>
+          <t>Diseña proyectos empresariales mediante análisis cuantitativo y metodologías de gestión, modelando escenarios organizacionales y asignando recursos, con rigor técnico, cumplimiento de objetivos y eficiencia operativa.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
@@ -1488,6 +1474,11 @@
       <c r="I45" s="12" t="n">
         <v>60.3</v>
       </c>
+      <c r="J45" s="22" t="inlineStr">
+        <is>
+          <t>Analiza mercados y entornos competitivos para estructurar estrategias de posicionamiento empresarial, utilizando segmentación y estudios de demanda, con diferenciación estratégica y generación de ventaja competitiva medible.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
@@ -1523,6 +1514,11 @@
       <c r="I46" s="8" t="n">
         <v>47.6</v>
       </c>
+      <c r="J46" s="22" t="inlineStr">
+        <is>
+          <t>Evalúa alternativas financieras y estructuras de inversión en organizaciones productivas o de servicios, aplicando herramientas de análisis económico y proyecciones financieras, con sustento cuantitativo, precisión técnica y control del riesgo.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
@@ -1558,6 +1554,11 @@
       <c r="I47" s="12" t="n">
         <v>46</v>
       </c>
+      <c r="J47" s="22" t="inlineStr">
+        <is>
+          <t>Formula estrategias y modelos de desarrollo empresarial en organizaciones públicas o privadas, con coherencia sistémica, visión directiva, capacidad de liderazgo estratégico y orientación a resultados verificables.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
@@ -1593,6 +1594,11 @@
       <c r="I48" s="8" t="n">
         <v>3.2</v>
       </c>
+      <c r="J48" s="22" t="inlineStr">
+        <is>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
@@ -1628,6 +1634,11 @@
       <c r="I49" s="12" t="n">
         <v>60.3</v>
       </c>
+      <c r="J49" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
@@ -1663,6 +1674,11 @@
       <c r="I50" s="8" t="n">
         <v>47.6</v>
       </c>
+      <c r="J50" s="22" t="inlineStr">
+        <is>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
@@ -1698,21 +1714,19 @@
       <c r="I51" s="12" t="n">
         <v>46</v>
       </c>
-    </row>
+      <c r="J51" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B53" s="6" t="n"/>
-      <c r="C53" s="6" t="n"/>
-      <c r="D53" s="6" t="n"/>
-      <c r="E53" s="6" t="n"/>
-      <c r="F53" s="6" t="n"/>
-      <c r="G53" s="6" t="n"/>
-      <c r="H53" s="6" t="n"/>
-      <c r="I53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
@@ -1757,30 +1771,18 @@
           <t>CE1 / CT1</t>
         </is>
       </c>
-      <c r="C56" s="16" t="n"/>
-      <c r="D56" s="16" t="n"/>
-      <c r="E56" s="16" t="n"/>
-      <c r="F56" s="16" t="n"/>
-      <c r="G56" s="16" t="n"/>
-      <c r="H56" s="16" t="n"/>
       <c r="I56" s="17" t="n">
         <v>31.7</v>
       </c>
     </row>
+    <row r="57"/>
+    <row r="58"/>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B59" s="6" t="n"/>
-      <c r="C59" s="6" t="n"/>
-      <c r="D59" s="6" t="n"/>
-      <c r="E59" s="6" t="n"/>
-      <c r="F59" s="6" t="n"/>
-      <c r="G59" s="6" t="n"/>
-      <c r="H59" s="6" t="n"/>
-      <c r="I59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
@@ -1825,12 +1827,6 @@
           <t>CE2 / CT2</t>
         </is>
       </c>
-      <c r="C62" s="16" t="n"/>
-      <c r="D62" s="16" t="n"/>
-      <c r="E62" s="16" t="n"/>
-      <c r="F62" s="16" t="n"/>
-      <c r="G62" s="16" t="n"/>
-      <c r="H62" s="16" t="n"/>
       <c r="I62" s="19" t="n">
         <v>95.2</v>
       </c>
@@ -1861,12 +1857,6 @@
           <t>CE2 / CT2</t>
         </is>
       </c>
-      <c r="C64" s="16" t="n"/>
-      <c r="D64" s="16" t="n"/>
-      <c r="E64" s="16" t="n"/>
-      <c r="F64" s="16" t="n"/>
-      <c r="G64" s="16" t="n"/>
-      <c r="H64" s="16" t="n"/>
       <c r="I64" s="19" t="n">
         <v>93.7</v>
       </c>
@@ -1897,12 +1887,6 @@
           <t>CE4 / CT4</t>
         </is>
       </c>
-      <c r="C66" s="16" t="n"/>
-      <c r="D66" s="16" t="n"/>
-      <c r="E66" s="16" t="n"/>
-      <c r="F66" s="16" t="n"/>
-      <c r="G66" s="16" t="n"/>
-      <c r="H66" s="16" t="n"/>
       <c r="I66" s="19" t="n">
         <v>92.09999999999999</v>
       </c>
@@ -1933,12 +1917,6 @@
           <t>CE4 / CT4</t>
         </is>
       </c>
-      <c r="C68" s="16" t="n"/>
-      <c r="D68" s="16" t="n"/>
-      <c r="E68" s="16" t="n"/>
-      <c r="F68" s="16" t="n"/>
-      <c r="G68" s="16" t="n"/>
-      <c r="H68" s="16" t="n"/>
       <c r="I68" s="19" t="n">
         <v>90.5</v>
       </c>
@@ -1969,12 +1947,6 @@
           <t>CE1 / CT1</t>
         </is>
       </c>
-      <c r="C70" s="16" t="n"/>
-      <c r="D70" s="16" t="n"/>
-      <c r="E70" s="16" t="n"/>
-      <c r="F70" s="16" t="n"/>
-      <c r="G70" s="16" t="n"/>
-      <c r="H70" s="16" t="n"/>
       <c r="I70" s="19" t="n">
         <v>90.5</v>
       </c>
@@ -1997,8 +1969,8 @@
   </sheetData>
   <mergeCells count="38">
     <mergeCell ref="A37:I37"/>
+    <mergeCell ref="B68:H68"/>
     <mergeCell ref="B65:H65"/>
-    <mergeCell ref="B68:H68"/>
     <mergeCell ref="B55:H55"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B30:H30"/>
@@ -2045,7 +2017,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:J66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2054,6 +2026,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2070,20 +2043,13 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>══ TA1 — 135 estudiantes ══</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -2091,14 +2057,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -2212,20 +2170,13 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -2273,6 +2224,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -2308,6 +2264,11 @@
       <c r="I12" s="8" t="n">
         <v>8.9</v>
       </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>Registra operaciones económicas de una entidad para la elaboración de estados financieros orientados a la toma de decisiones conforme a la normativa contable.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -2343,6 +2304,11 @@
       <c r="I13" s="12" t="n">
         <v>14.8</v>
       </c>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>Calcula las obligaciones tributarias de personas naturales y jurídicas con base a la legislación tributaria garantizando la exactitud de las declaraciones.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -2378,6 +2344,11 @@
       <c r="I14" s="8" t="n">
         <v>9.6</v>
       </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona los recursos financieros de las organizaciones, garantizando la adecuada planificación y control financiero.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -2413,6 +2384,11 @@
       <c r="I15" s="12" t="n">
         <v>14.8</v>
       </c>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>Analiza situaciones profesionales y toma decisiones fundamentadas considerando impactos sociales, ambientales, económicos y tecnológicos, actuando con responsabilidad, integridad y compromiso con el desarrollo sostenible en contextos locales y globales.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -2448,6 +2424,11 @@
       <c r="I16" s="8" t="n">
         <v>21.5</v>
       </c>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas con claridad y sustento técnico, y colabora eficazmente en equipos diversos e interdisciplinarios, contribuyendo activamente a la construcción de soluciones en entornos profesionales, multiculturales y digitales.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -2483,6 +2464,11 @@
       <c r="I17" s="12" t="n">
         <v>25.9</v>
       </c>
+      <c r="J17" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona información y conocimiento con rigor metodológico, actualizándose de manera autónoma y aplicando nuevos saberes para resolver problemas complejos en contextos dinámicos y cambiantes.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -2518,21 +2504,19 @@
       <c r="I18" s="8" t="n">
         <v>11.9</v>
       </c>
-    </row>
+      <c r="J18" s="22" t="inlineStr">
+        <is>
+          <t>Integra tecnologías digitales, análisis de datos y herramientas emergentes de manera crítica, ética y estratégica para generar soluciones pertinentes y sostenibles en contextos profesionales y sociales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -2577,12 +2561,6 @@
           <t>CE1 / CT1</t>
         </is>
       </c>
-      <c r="C23" s="16" t="n"/>
-      <c r="D23" s="16" t="n"/>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="16" t="n"/>
-      <c r="G23" s="16" t="n"/>
-      <c r="H23" s="16" t="n"/>
       <c r="I23" s="17" t="n">
         <v>40</v>
       </c>
@@ -2613,30 +2591,18 @@
           <t>CE2 / CT3</t>
         </is>
       </c>
-      <c r="C25" s="16" t="n"/>
-      <c r="D25" s="16" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="16" t="n"/>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="16" t="n"/>
       <c r="I25" s="17" t="n">
         <v>45.9</v>
       </c>
     </row>
+    <row r="26"/>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B28" s="6" t="n"/>
-      <c r="C28" s="6" t="n"/>
-      <c r="D28" s="6" t="n"/>
-      <c r="E28" s="6" t="n"/>
-      <c r="F28" s="6" t="n"/>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
@@ -2670,20 +2636,14 @@
         <v>94.8</v>
       </c>
     </row>
+    <row r="31"/>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
           <t>══ TA2 — 86 estudiantes ══</t>
         </is>
       </c>
-      <c r="B33" s="4" t="n"/>
-      <c r="C33" s="4" t="n"/>
-      <c r="D33" s="4" t="n"/>
-      <c r="E33" s="4" t="n"/>
-      <c r="F33" s="4" t="n"/>
-      <c r="G33" s="4" t="n"/>
-      <c r="H33" s="4" t="n"/>
-      <c r="I33" s="4" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2691,14 +2651,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B34" s="6" t="n"/>
-      <c r="C34" s="6" t="n"/>
-      <c r="D34" s="6" t="n"/>
-      <c r="E34" s="6" t="n"/>
-      <c r="F34" s="6" t="n"/>
-      <c r="G34" s="6" t="n"/>
-      <c r="H34" s="6" t="n"/>
-      <c r="I34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
@@ -2812,20 +2764,13 @@
         </is>
       </c>
     </row>
+    <row r="38"/>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B39" s="6" t="n"/>
-      <c r="C39" s="6" t="n"/>
-      <c r="D39" s="6" t="n"/>
-      <c r="E39" s="6" t="n"/>
-      <c r="F39" s="6" t="n"/>
-      <c r="G39" s="6" t="n"/>
-      <c r="H39" s="6" t="n"/>
-      <c r="I39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
@@ -2873,6 +2818,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J40" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -2908,6 +2858,11 @@
       <c r="I41" s="8" t="n">
         <v>11.6</v>
       </c>
+      <c r="J41" s="22" t="inlineStr">
+        <is>
+          <t>Registra operaciones económicas de una entidad para la elaboración de estados financieros orientados a la toma de decisiones conforme a la normativa contable.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -2943,6 +2898,11 @@
       <c r="I42" s="12" t="n">
         <v>22.1</v>
       </c>
+      <c r="J42" s="22" t="inlineStr">
+        <is>
+          <t>Calcula las obligaciones tributarias de personas naturales y jurídicas con base a la legislación tributaria garantizando la exactitud de las declaraciones.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
@@ -2978,6 +2938,11 @@
       <c r="I43" s="8" t="n">
         <v>17.4</v>
       </c>
+      <c r="J43" s="22" t="inlineStr">
+        <is>
+          <t>Aplica procedimientos de auditoría en el ámbito empresarial para evaluar el control interno y verificar la transparencia de la información financiera, conforme a normas internacionales de auditoría.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
@@ -3013,6 +2978,11 @@
       <c r="I44" s="12" t="n">
         <v>18.6</v>
       </c>
+      <c r="J44" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona los recursos financieros de las organizaciones, garantizando la adecuada planificación y control financiero.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
@@ -3048,6 +3018,11 @@
       <c r="I45" s="8" t="n">
         <v>12.8</v>
       </c>
+      <c r="J45" s="22" t="inlineStr">
+        <is>
+          <t>Analiza situaciones profesionales y toma decisiones fundamentadas considerando impactos sociales, ambientales, económicos y tecnológicos, actuando con responsabilidad, integridad y compromiso con el desarrollo sostenible en contextos locales y globales.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
@@ -3083,6 +3058,11 @@
       <c r="I46" s="12" t="n">
         <v>18.6</v>
       </c>
+      <c r="J46" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas con claridad y sustento técnico, y colabora eficazmente en equipos diversos e interdisciplinarios, contribuyendo activamente a la construcción de soluciones en entornos profesionales, multiculturales y digitales.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
@@ -3118,6 +3098,11 @@
       <c r="I47" s="8" t="n">
         <v>20.9</v>
       </c>
+      <c r="J47" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona información y conocimiento con rigor metodológico, actualizándose de manera autónoma y aplicando nuevos saberes para resolver problemas complejos en contextos dinámicos y cambiantes.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
@@ -3153,21 +3138,19 @@
       <c r="I48" s="12" t="n">
         <v>15.1</v>
       </c>
-    </row>
+      <c r="J48" s="22" t="inlineStr">
+        <is>
+          <t>Integra tecnologías digitales, análisis de datos y herramientas emergentes de manera crítica, ética y estratégica para generar soluciones pertinentes y sostenibles en contextos profesionales y sociales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49"/>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B50" s="6" t="n"/>
-      <c r="C50" s="6" t="n"/>
-      <c r="D50" s="6" t="n"/>
-      <c r="E50" s="6" t="n"/>
-      <c r="F50" s="6" t="n"/>
-      <c r="G50" s="6" t="n"/>
-      <c r="H50" s="6" t="n"/>
-      <c r="I50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
@@ -3212,12 +3195,6 @@
           <t>CE1 / CT1</t>
         </is>
       </c>
-      <c r="C53" s="16" t="n"/>
-      <c r="D53" s="16" t="n"/>
-      <c r="E53" s="16" t="n"/>
-      <c r="F53" s="16" t="n"/>
-      <c r="G53" s="16" t="n"/>
-      <c r="H53" s="16" t="n"/>
       <c r="I53" s="17" t="n">
         <v>30.2</v>
       </c>
@@ -3248,30 +3225,18 @@
           <t>CE2 / CT4</t>
         </is>
       </c>
-      <c r="C55" s="16" t="n"/>
-      <c r="D55" s="16" t="n"/>
-      <c r="E55" s="16" t="n"/>
-      <c r="F55" s="16" t="n"/>
-      <c r="G55" s="16" t="n"/>
-      <c r="H55" s="16" t="n"/>
       <c r="I55" s="17" t="n">
         <v>38.4</v>
       </c>
     </row>
+    <row r="56"/>
+    <row r="57"/>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B58" s="6" t="n"/>
-      <c r="C58" s="6" t="n"/>
-      <c r="D58" s="6" t="n"/>
-      <c r="E58" s="6" t="n"/>
-      <c r="F58" s="6" t="n"/>
-      <c r="G58" s="6" t="n"/>
-      <c r="H58" s="6" t="n"/>
-      <c r="I58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
@@ -3316,12 +3281,6 @@
           <t>CE2 / CT1</t>
         </is>
       </c>
-      <c r="C61" s="16" t="n"/>
-      <c r="D61" s="16" t="n"/>
-      <c r="E61" s="16" t="n"/>
-      <c r="F61" s="16" t="n"/>
-      <c r="G61" s="16" t="n"/>
-      <c r="H61" s="16" t="n"/>
       <c r="I61" s="19" t="n">
         <v>98.8</v>
       </c>
@@ -3352,12 +3311,6 @@
           <t>CE4 / CT2</t>
         </is>
       </c>
-      <c r="C63" s="16" t="n"/>
-      <c r="D63" s="16" t="n"/>
-      <c r="E63" s="16" t="n"/>
-      <c r="F63" s="16" t="n"/>
-      <c r="G63" s="16" t="n"/>
-      <c r="H63" s="16" t="n"/>
       <c r="I63" s="19" t="n">
         <v>98.8</v>
       </c>
@@ -3388,12 +3341,6 @@
           <t>CE4 / CT3</t>
         </is>
       </c>
-      <c r="C65" s="16" t="n"/>
-      <c r="D65" s="16" t="n"/>
-      <c r="E65" s="16" t="n"/>
-      <c r="F65" s="16" t="n"/>
-      <c r="G65" s="16" t="n"/>
-      <c r="H65" s="16" t="n"/>
       <c r="I65" s="19" t="n">
         <v>96.5</v>
       </c>
@@ -3460,7 +3407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:J64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3469,6 +3416,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3485,20 +3433,13 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>══ TA1 — 120 estudiantes ══</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -3506,14 +3447,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -3627,20 +3560,13 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -3688,6 +3614,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -3723,6 +3654,11 @@
       <c r="I12" s="8" t="n">
         <v>56.7</v>
       </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>Analiza fenómenos económicos mediante el estudio del comportamiento de agentes y la dinámica de variables agregadas, con fundamento en los principios teóricos y metodológicos de la ciencia económica.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -3758,6 +3694,11 @@
       <c r="I13" s="12" t="n">
         <v>0.8</v>
       </c>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>Construye modelos econométricos a partir de datos económicos, con rigor metodológico, capacidad explicativa y predictiva.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -3793,6 +3734,11 @@
       <c r="I14" s="8" t="n">
         <v>11.7</v>
       </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>Evalúa el desempeño económico y financiero de organizaciones y sectores productivos a través de herramientas e indicadores financieros, con precisión técnica y visión integral.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -3828,6 +3774,11 @@
       <c r="I15" s="12" t="n">
         <v>16.7</v>
       </c>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -3863,6 +3814,11 @@
       <c r="I16" s="8" t="n">
         <v>0.8</v>
       </c>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -3898,6 +3854,11 @@
       <c r="I17" s="12" t="n">
         <v>27.5</v>
       </c>
+      <c r="J17" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -3933,21 +3894,19 @@
       <c r="I18" s="8" t="n">
         <v>4.2</v>
       </c>
-    </row>
+      <c r="J18" s="22" t="inlineStr">
+        <is>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -3992,12 +3951,6 @@
           <t>CE2 / CT2</t>
         </is>
       </c>
-      <c r="C23" s="16" t="n"/>
-      <c r="D23" s="16" t="n"/>
-      <c r="E23" s="16" t="n"/>
-      <c r="F23" s="16" t="n"/>
-      <c r="G23" s="16" t="n"/>
-      <c r="H23" s="16" t="n"/>
       <c r="I23" s="17" t="n">
         <v>15</v>
       </c>
@@ -4028,12 +3981,6 @@
           <t>CE3 / CT4</t>
         </is>
       </c>
-      <c r="C25" s="16" t="n"/>
-      <c r="D25" s="16" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="16" t="n"/>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="16" t="n"/>
       <c r="I25" s="17" t="n">
         <v>19.2</v>
       </c>
@@ -4064,12 +4011,6 @@
           <t>CE3 / CT4</t>
         </is>
       </c>
-      <c r="C27" s="16" t="n"/>
-      <c r="D27" s="16" t="n"/>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="16" t="n"/>
-      <c r="G27" s="16" t="n"/>
-      <c r="H27" s="16" t="n"/>
       <c r="I27" s="17" t="n">
         <v>34.2</v>
       </c>
@@ -4100,30 +4041,18 @@
           <t>CE3 / CT1</t>
         </is>
       </c>
-      <c r="C29" s="16" t="n"/>
-      <c r="D29" s="16" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="16" t="n"/>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="16" t="n"/>
       <c r="I29" s="17" t="n">
         <v>47.5</v>
       </c>
     </row>
+    <row r="30"/>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B32" s="6" t="n"/>
-      <c r="C32" s="6" t="n"/>
-      <c r="D32" s="6" t="n"/>
-      <c r="E32" s="6" t="n"/>
-      <c r="F32" s="6" t="n"/>
-      <c r="G32" s="6" t="n"/>
-      <c r="H32" s="6" t="n"/>
-      <c r="I32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
@@ -4168,12 +4097,6 @@
           <t>CE1 / CT3</t>
         </is>
       </c>
-      <c r="C35" s="16" t="n"/>
-      <c r="D35" s="16" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="16" t="n"/>
-      <c r="G35" s="16" t="n"/>
-      <c r="H35" s="16" t="n"/>
       <c r="I35" s="19" t="n">
         <v>91.7</v>
       </c>
@@ -4193,20 +4116,14 @@
         <v>90</v>
       </c>
     </row>
+    <row r="37"/>
+    <row r="38"/>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
           <t>══ TA2 — 64 estudiantes ══</t>
         </is>
       </c>
-      <c r="B39" s="4" t="n"/>
-      <c r="C39" s="4" t="n"/>
-      <c r="D39" s="4" t="n"/>
-      <c r="E39" s="4" t="n"/>
-      <c r="F39" s="4" t="n"/>
-      <c r="G39" s="4" t="n"/>
-      <c r="H39" s="4" t="n"/>
-      <c r="I39" s="4" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -4214,14 +4131,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="6" t="n"/>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="6" t="n"/>
-      <c r="H40" s="6" t="n"/>
-      <c r="I40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -4335,20 +4244,13 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B45" s="6" t="n"/>
-      <c r="C45" s="6" t="n"/>
-      <c r="D45" s="6" t="n"/>
-      <c r="E45" s="6" t="n"/>
-      <c r="F45" s="6" t="n"/>
-      <c r="G45" s="6" t="n"/>
-      <c r="H45" s="6" t="n"/>
-      <c r="I45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
@@ -4396,6 +4298,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J46" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
@@ -4431,6 +4338,11 @@
       <c r="I47" s="8" t="n">
         <v>46.9</v>
       </c>
+      <c r="J47" s="22" t="inlineStr">
+        <is>
+          <t>Analiza fenómenos económicos mediante el estudio del comportamiento de agentes y la dinámica de variables agregadas, con fundamento en los principios teóricos y metodológicos de la ciencia económica.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
@@ -4466,6 +4378,11 @@
       <c r="I48" s="12" t="n">
         <v>7.8</v>
       </c>
+      <c r="J48" s="22" t="inlineStr">
+        <is>
+          <t>Construye modelos econométricos a partir de datos económicos, con rigor metodológico, capacidad explicativa y predictiva.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
@@ -4501,6 +4418,11 @@
       <c r="I49" s="8" t="n">
         <v>42.2</v>
       </c>
+      <c r="J49" s="22" t="inlineStr">
+        <is>
+          <t>Evalúa el desempeño económico y financiero de organizaciones y sectores productivos a través de herramientas e indicadores financieros, con precisión técnica y visión integral.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
@@ -4536,6 +4458,11 @@
       <c r="I50" s="12" t="n">
         <v>6.2</v>
       </c>
+      <c r="J50" s="22" t="inlineStr">
+        <is>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
@@ -4571,6 +4498,11 @@
       <c r="I51" s="8" t="n">
         <v>6.2</v>
       </c>
+      <c r="J51" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
@@ -4606,6 +4538,11 @@
       <c r="I52" s="12" t="n">
         <v>18.8</v>
       </c>
+      <c r="J52" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
@@ -4641,21 +4578,19 @@
       <c r="I53" s="8" t="n">
         <v>82.8</v>
       </c>
-    </row>
+      <c r="J53" s="22" t="inlineStr">
+        <is>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54"/>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="6" t="n"/>
-      <c r="D55" s="6" t="n"/>
-      <c r="E55" s="6" t="n"/>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="6" t="n"/>
-      <c r="H55" s="6" t="n"/>
-      <c r="I55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -4700,12 +4635,6 @@
           <t>CE2 / CT1 / CT2</t>
         </is>
       </c>
-      <c r="C58" s="16" t="n"/>
-      <c r="D58" s="16" t="n"/>
-      <c r="E58" s="16" t="n"/>
-      <c r="F58" s="16" t="n"/>
-      <c r="G58" s="16" t="n"/>
-      <c r="H58" s="16" t="n"/>
       <c r="I58" s="17" t="n">
         <v>12.5</v>
       </c>
@@ -4725,20 +4654,14 @@
         <v>21.9</v>
       </c>
     </row>
+    <row r="60"/>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B62" s="6" t="n"/>
-      <c r="C62" s="6" t="n"/>
-      <c r="D62" s="6" t="n"/>
-      <c r="E62" s="6" t="n"/>
-      <c r="F62" s="6" t="n"/>
-      <c r="G62" s="6" t="n"/>
-      <c r="H62" s="6" t="n"/>
-      <c r="I62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -4790,8 +4713,8 @@
     <mergeCell ref="B59:H59"/>
     <mergeCell ref="A4:I4"/>
     <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A62:I62"/>
     <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A62:I62"/>
     <mergeCell ref="B22:H22"/>
     <mergeCell ref="B27:H27"/>
     <mergeCell ref="A10:I10"/>
@@ -4818,7 +4741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I70"/>
+  <dimension ref="A1:J70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -4827,6 +4750,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4843,20 +4767,13 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>══ TA1 — 154 estudiantes ══</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -4864,14 +4781,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -4985,20 +4894,13 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -5046,6 +4948,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -5081,6 +4988,11 @@
       <c r="I12" s="8" t="n">
         <v>61</v>
       </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>Analiza fenómenos, modelos e información económica, para comprender la interacción entre los agentes económicos, bajo el criterio de eficiencia.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -5116,6 +5028,11 @@
       <c r="I13" s="12" t="n">
         <v>61</v>
       </c>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>Aplica herramientas cuantitativas, estadísticas y econométricas para construir escenarios económicos sustentados en la teoría económica, que apoyen la toma de decisiones en contextos de incertidumbre.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -5151,6 +5068,11 @@
       <c r="I14" s="8" t="n">
         <v>61</v>
       </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -5186,21 +5108,19 @@
       <c r="I15" s="12" t="n">
         <v>61</v>
       </c>
-    </row>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B17" s="6" t="n"/>
-      <c r="C17" s="6" t="n"/>
-      <c r="D17" s="6" t="n"/>
-      <c r="E17" s="6" t="n"/>
-      <c r="F17" s="6" t="n"/>
-      <c r="G17" s="6" t="n"/>
-      <c r="H17" s="6" t="n"/>
-      <c r="I17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
@@ -5226,20 +5146,14 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B22" s="6" t="n"/>
-      <c r="C22" s="6" t="n"/>
-      <c r="D22" s="6" t="n"/>
-      <c r="E22" s="6" t="n"/>
-      <c r="F22" s="6" t="n"/>
-      <c r="G22" s="6" t="n"/>
-      <c r="H22" s="6" t="n"/>
-      <c r="I22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
@@ -5284,12 +5198,6 @@
           <t>CE2 / CT3</t>
         </is>
       </c>
-      <c r="C25" s="16" t="n"/>
-      <c r="D25" s="16" t="n"/>
-      <c r="E25" s="16" t="n"/>
-      <c r="F25" s="16" t="n"/>
-      <c r="G25" s="16" t="n"/>
-      <c r="H25" s="16" t="n"/>
       <c r="I25" s="19" t="n">
         <v>95.5</v>
       </c>
@@ -5320,12 +5228,6 @@
           <t>CE2 / CT3</t>
         </is>
       </c>
-      <c r="C27" s="16" t="n"/>
-      <c r="D27" s="16" t="n"/>
-      <c r="E27" s="16" t="n"/>
-      <c r="F27" s="16" t="n"/>
-      <c r="G27" s="16" t="n"/>
-      <c r="H27" s="16" t="n"/>
       <c r="I27" s="19" t="n">
         <v>92.2</v>
       </c>
@@ -5356,12 +5258,6 @@
           <t>CE2 / CT3</t>
         </is>
       </c>
-      <c r="C29" s="16" t="n"/>
-      <c r="D29" s="16" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="16" t="n"/>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="16" t="n"/>
       <c r="I29" s="19" t="n">
         <v>90.90000000000001</v>
       </c>
@@ -5392,30 +5288,18 @@
           <t>CE1 / CT4</t>
         </is>
       </c>
-      <c r="C31" s="16" t="n"/>
-      <c r="D31" s="16" t="n"/>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="16" t="n"/>
-      <c r="G31" s="16" t="n"/>
-      <c r="H31" s="16" t="n"/>
       <c r="I31" s="19" t="n">
         <v>90.3</v>
       </c>
     </row>
+    <row r="32"/>
+    <row r="33"/>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
           <t>══ TA2 — 337 estudiantes ══</t>
         </is>
       </c>
-      <c r="B34" s="4" t="n"/>
-      <c r="C34" s="4" t="n"/>
-      <c r="D34" s="4" t="n"/>
-      <c r="E34" s="4" t="n"/>
-      <c r="F34" s="4" t="n"/>
-      <c r="G34" s="4" t="n"/>
-      <c r="H34" s="4" t="n"/>
-      <c r="I34" s="4" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -5423,14 +5307,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B35" s="6" t="n"/>
-      <c r="C35" s="6" t="n"/>
-      <c r="D35" s="6" t="n"/>
-      <c r="E35" s="6" t="n"/>
-      <c r="F35" s="6" t="n"/>
-      <c r="G35" s="6" t="n"/>
-      <c r="H35" s="6" t="n"/>
-      <c r="I35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -5544,20 +5420,13 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B40" s="6" t="n"/>
-      <c r="C40" s="6" t="n"/>
-      <c r="D40" s="6" t="n"/>
-      <c r="E40" s="6" t="n"/>
-      <c r="F40" s="6" t="n"/>
-      <c r="G40" s="6" t="n"/>
-      <c r="H40" s="6" t="n"/>
-      <c r="I40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
@@ -5605,6 +5474,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J41" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
@@ -5640,6 +5514,11 @@
       <c r="I42" s="8" t="n">
         <v>92.90000000000001</v>
       </c>
+      <c r="J42" s="22" t="inlineStr">
+        <is>
+          <t>Evalúa políticas públicas, planes, programas y proyectos económicos para proponer soluciones a problemáticas económicas, considerando los sectores público y privado.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -5675,6 +5554,11 @@
       <c r="I43" s="12" t="n">
         <v>81.90000000000001</v>
       </c>
+      <c r="J43" s="22" t="inlineStr">
+        <is>
+          <t>Desarrolla investigación económica aplicada para proponer soluciones a problemas económicos y sociales vinculados al entorno local y global.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
@@ -5710,6 +5594,11 @@
       <c r="I44" s="8" t="n">
         <v>92.90000000000001</v>
       </c>
+      <c r="J44" s="22" t="inlineStr">
+        <is>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
@@ -5745,21 +5634,19 @@
       <c r="I45" s="12" t="n">
         <v>81.90000000000001</v>
       </c>
-    </row>
+      <c r="J45" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B47" s="6" t="n"/>
-      <c r="C47" s="6" t="n"/>
-      <c r="D47" s="6" t="n"/>
-      <c r="E47" s="6" t="n"/>
-      <c r="F47" s="6" t="n"/>
-      <c r="G47" s="6" t="n"/>
-      <c r="H47" s="6" t="n"/>
-      <c r="I47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
@@ -5785,20 +5672,14 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B52" s="6" t="n"/>
-      <c r="C52" s="6" t="n"/>
-      <c r="D52" s="6" t="n"/>
-      <c r="E52" s="6" t="n"/>
-      <c r="F52" s="6" t="n"/>
-      <c r="G52" s="6" t="n"/>
-      <c r="H52" s="6" t="n"/>
-      <c r="I52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
@@ -5843,12 +5724,6 @@
           <t>CE3 / CT1</t>
         </is>
       </c>
-      <c r="C55" s="16" t="n"/>
-      <c r="D55" s="16" t="n"/>
-      <c r="E55" s="16" t="n"/>
-      <c r="F55" s="16" t="n"/>
-      <c r="G55" s="16" t="n"/>
-      <c r="H55" s="16" t="n"/>
       <c r="I55" s="19" t="n">
         <v>98.2</v>
       </c>
@@ -5879,12 +5754,6 @@
           <t>CE3 / CT1</t>
         </is>
       </c>
-      <c r="C57" s="16" t="n"/>
-      <c r="D57" s="16" t="n"/>
-      <c r="E57" s="16" t="n"/>
-      <c r="F57" s="16" t="n"/>
-      <c r="G57" s="16" t="n"/>
-      <c r="H57" s="16" t="n"/>
       <c r="I57" s="19" t="n">
         <v>97.90000000000001</v>
       </c>
@@ -5915,12 +5784,6 @@
           <t>CE3 / CT1</t>
         </is>
       </c>
-      <c r="C59" s="16" t="n"/>
-      <c r="D59" s="16" t="n"/>
-      <c r="E59" s="16" t="n"/>
-      <c r="F59" s="16" t="n"/>
-      <c r="G59" s="16" t="n"/>
-      <c r="H59" s="16" t="n"/>
       <c r="I59" s="19" t="n">
         <v>97.3</v>
       </c>
@@ -5951,12 +5814,6 @@
           <t>CE3 / CT1</t>
         </is>
       </c>
-      <c r="C61" s="16" t="n"/>
-      <c r="D61" s="16" t="n"/>
-      <c r="E61" s="16" t="n"/>
-      <c r="F61" s="16" t="n"/>
-      <c r="G61" s="16" t="n"/>
-      <c r="H61" s="16" t="n"/>
       <c r="I61" s="19" t="n">
         <v>97</v>
       </c>
@@ -5987,12 +5844,6 @@
           <t>CE3 / CT1</t>
         </is>
       </c>
-      <c r="C63" s="16" t="n"/>
-      <c r="D63" s="16" t="n"/>
-      <c r="E63" s="16" t="n"/>
-      <c r="F63" s="16" t="n"/>
-      <c r="G63" s="16" t="n"/>
-      <c r="H63" s="16" t="n"/>
       <c r="I63" s="19" t="n">
         <v>96.09999999999999</v>
       </c>
@@ -6023,12 +5874,6 @@
           <t>CE4 / CT2</t>
         </is>
       </c>
-      <c r="C65" s="16" t="n"/>
-      <c r="D65" s="16" t="n"/>
-      <c r="E65" s="16" t="n"/>
-      <c r="F65" s="16" t="n"/>
-      <c r="G65" s="16" t="n"/>
-      <c r="H65" s="16" t="n"/>
       <c r="I65" s="19" t="n">
         <v>95.3</v>
       </c>
@@ -6059,12 +5904,6 @@
           <t>CE3 / CT1</t>
         </is>
       </c>
-      <c r="C67" s="16" t="n"/>
-      <c r="D67" s="16" t="n"/>
-      <c r="E67" s="16" t="n"/>
-      <c r="F67" s="16" t="n"/>
-      <c r="G67" s="16" t="n"/>
-      <c r="H67" s="16" t="n"/>
       <c r="I67" s="19" t="n">
         <v>93.8</v>
       </c>
@@ -6095,12 +5934,6 @@
           <t>CE4 / CT2</t>
         </is>
       </c>
-      <c r="C69" s="16" t="n"/>
-      <c r="D69" s="16" t="n"/>
-      <c r="E69" s="16" t="n"/>
-      <c r="F69" s="16" t="n"/>
-      <c r="G69" s="16" t="n"/>
-      <c r="H69" s="16" t="n"/>
       <c r="I69" s="19" t="n">
         <v>93.5</v>
       </c>
@@ -6123,8 +5956,8 @@
   </sheetData>
   <mergeCells count="43">
     <mergeCell ref="H38:I38"/>
+    <mergeCell ref="B68:H68"/>
     <mergeCell ref="B65:H65"/>
-    <mergeCell ref="B68:H68"/>
     <mergeCell ref="B55:H55"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B30:H30"/>
@@ -6176,7 +6009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6185,6 +6018,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6201,20 +6035,13 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>══ TA1 — 60 estudiantes ══</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -6222,14 +6049,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -6343,20 +6162,13 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -6404,6 +6216,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -6439,6 +6256,11 @@
       <c r="I12" s="8" t="n">
         <v>100</v>
       </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>Diseña productos, experiencias y servicios turísticos en contextos territoriales y organizacionales, garantizando innovación, sostenibilidad y estándares de calidad internacional.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -6474,6 +6296,11 @@
       <c r="I13" s="12" t="n">
         <v>100</v>
       </c>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>Formula estrategias de planificación y comercialización turística en destinos y organizaciones del sector, asegurando competitividad y posicionamiento en el mercado.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -6509,6 +6336,11 @@
       <c r="I14" s="8" t="n">
         <v>100</v>
       </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>Optimiza procesos de gestión y operación turística en empresas y emprendimientos del sector, garantizando eficiencia, rentabilidad y mejora continua.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -6544,6 +6376,11 @@
       <c r="I15" s="12" t="n">
         <v>100</v>
       </c>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>Evalúa proyectos y servicios turísticos en función del análisis de mercado y segmentación de la demanda, fundamentando decisiones estratégicas sostenibles.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -6579,6 +6416,11 @@
       <c r="I16" s="8" t="n">
         <v>100</v>
       </c>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -6614,6 +6456,11 @@
       <c r="I17" s="12" t="n">
         <v>100</v>
       </c>
+      <c r="J17" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -6649,6 +6496,11 @@
       <c r="I18" s="8" t="n">
         <v>100</v>
       </c>
+      <c r="J18" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -6684,21 +6536,19 @@
       <c r="I19" s="12" t="n">
         <v>100</v>
       </c>
-    </row>
+      <c r="J19" s="22" t="inlineStr">
+        <is>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B21" s="6" t="n"/>
-      <c r="C21" s="6" t="n"/>
-      <c r="D21" s="6" t="n"/>
-      <c r="E21" s="6" t="n"/>
-      <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
-      <c r="H21" s="6" t="n"/>
-      <c r="I21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
@@ -6724,20 +6574,14 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B26" s="6" t="n"/>
-      <c r="C26" s="6" t="n"/>
-      <c r="D26" s="6" t="n"/>
-      <c r="E26" s="6" t="n"/>
-      <c r="F26" s="6" t="n"/>
-      <c r="G26" s="6" t="n"/>
-      <c r="H26" s="6" t="n"/>
-      <c r="I26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -6782,12 +6626,6 @@
           <t>CE1 / CT4</t>
         </is>
       </c>
-      <c r="C29" s="16" t="n"/>
-      <c r="D29" s="16" t="n"/>
-      <c r="E29" s="16" t="n"/>
-      <c r="F29" s="16" t="n"/>
-      <c r="G29" s="16" t="n"/>
-      <c r="H29" s="16" t="n"/>
       <c r="I29" s="19" t="n">
         <v>100</v>
       </c>
@@ -6818,12 +6656,6 @@
           <t>CE1 / CT4</t>
         </is>
       </c>
-      <c r="C31" s="16" t="n"/>
-      <c r="D31" s="16" t="n"/>
-      <c r="E31" s="16" t="n"/>
-      <c r="F31" s="16" t="n"/>
-      <c r="G31" s="16" t="n"/>
-      <c r="H31" s="16" t="n"/>
       <c r="I31" s="19" t="n">
         <v>100</v>
       </c>
@@ -6854,12 +6686,6 @@
           <t>CE1 / CT4</t>
         </is>
       </c>
-      <c r="C33" s="16" t="n"/>
-      <c r="D33" s="16" t="n"/>
-      <c r="E33" s="16" t="n"/>
-      <c r="F33" s="16" t="n"/>
-      <c r="G33" s="16" t="n"/>
-      <c r="H33" s="16" t="n"/>
       <c r="I33" s="19" t="n">
         <v>100</v>
       </c>
@@ -6890,12 +6716,6 @@
           <t>CE2 / CT2</t>
         </is>
       </c>
-      <c r="C35" s="16" t="n"/>
-      <c r="D35" s="16" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="16" t="n"/>
-      <c r="G35" s="16" t="n"/>
-      <c r="H35" s="16" t="n"/>
       <c r="I35" s="19" t="n">
         <v>100</v>
       </c>
@@ -6926,12 +6746,6 @@
           <t>CE2 / CT2</t>
         </is>
       </c>
-      <c r="C37" s="16" t="n"/>
-      <c r="D37" s="16" t="n"/>
-      <c r="E37" s="16" t="n"/>
-      <c r="F37" s="16" t="n"/>
-      <c r="G37" s="16" t="n"/>
-      <c r="H37" s="16" t="n"/>
       <c r="I37" s="19" t="n">
         <v>100</v>
       </c>
@@ -6962,12 +6776,6 @@
           <t>CE2 / CT2</t>
         </is>
       </c>
-      <c r="C39" s="16" t="n"/>
-      <c r="D39" s="16" t="n"/>
-      <c r="E39" s="16" t="n"/>
-      <c r="F39" s="16" t="n"/>
-      <c r="G39" s="16" t="n"/>
-      <c r="H39" s="16" t="n"/>
       <c r="I39" s="19" t="n">
         <v>100</v>
       </c>
@@ -6998,12 +6806,6 @@
           <t>CE3 / CT3</t>
         </is>
       </c>
-      <c r="C41" s="16" t="n"/>
-      <c r="D41" s="16" t="n"/>
-      <c r="E41" s="16" t="n"/>
-      <c r="F41" s="16" t="n"/>
-      <c r="G41" s="16" t="n"/>
-      <c r="H41" s="16" t="n"/>
       <c r="I41" s="19" t="n">
         <v>100</v>
       </c>
@@ -7034,12 +6836,6 @@
           <t>CE3 / CT3</t>
         </is>
       </c>
-      <c r="C43" s="16" t="n"/>
-      <c r="D43" s="16" t="n"/>
-      <c r="E43" s="16" t="n"/>
-      <c r="F43" s="16" t="n"/>
-      <c r="G43" s="16" t="n"/>
-      <c r="H43" s="16" t="n"/>
       <c r="I43" s="19" t="n">
         <v>100</v>
       </c>
@@ -7070,12 +6866,6 @@
           <t>CE3 / CT3</t>
         </is>
       </c>
-      <c r="C45" s="16" t="n"/>
-      <c r="D45" s="16" t="n"/>
-      <c r="E45" s="16" t="n"/>
-      <c r="F45" s="16" t="n"/>
-      <c r="G45" s="16" t="n"/>
-      <c r="H45" s="16" t="n"/>
       <c r="I45" s="19" t="n">
         <v>100</v>
       </c>
@@ -7106,12 +6896,6 @@
           <t>CE4 / CT1</t>
         </is>
       </c>
-      <c r="C47" s="16" t="n"/>
-      <c r="D47" s="16" t="n"/>
-      <c r="E47" s="16" t="n"/>
-      <c r="F47" s="16" t="n"/>
-      <c r="G47" s="16" t="n"/>
-      <c r="H47" s="16" t="n"/>
       <c r="I47" s="19" t="n">
         <v>100</v>
       </c>
@@ -7142,12 +6926,6 @@
           <t>CE4 / CT1</t>
         </is>
       </c>
-      <c r="C49" s="16" t="n"/>
-      <c r="D49" s="16" t="n"/>
-      <c r="E49" s="16" t="n"/>
-      <c r="F49" s="16" t="n"/>
-      <c r="G49" s="16" t="n"/>
-      <c r="H49" s="16" t="n"/>
       <c r="I49" s="19" t="n">
         <v>100</v>
       </c>
@@ -7178,30 +6956,18 @@
           <t>CE4 / CT1</t>
         </is>
       </c>
-      <c r="C51" s="16" t="n"/>
-      <c r="D51" s="16" t="n"/>
-      <c r="E51" s="16" t="n"/>
-      <c r="F51" s="16" t="n"/>
-      <c r="G51" s="16" t="n"/>
-      <c r="H51" s="16" t="n"/>
       <c r="I51" s="19" t="n">
         <v>100</v>
       </c>
     </row>
+    <row r="52"/>
+    <row r="53"/>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
           <t>══ TA2 — 19 estudiantes ══</t>
         </is>
       </c>
-      <c r="B54" s="4" t="n"/>
-      <c r="C54" s="4" t="n"/>
-      <c r="D54" s="4" t="n"/>
-      <c r="E54" s="4" t="n"/>
-      <c r="F54" s="4" t="n"/>
-      <c r="G54" s="4" t="n"/>
-      <c r="H54" s="4" t="n"/>
-      <c r="I54" s="4" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
@@ -7209,14 +6975,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B55" s="6" t="n"/>
-      <c r="C55" s="6" t="n"/>
-      <c r="D55" s="6" t="n"/>
-      <c r="E55" s="6" t="n"/>
-      <c r="F55" s="6" t="n"/>
-      <c r="G55" s="6" t="n"/>
-      <c r="H55" s="6" t="n"/>
-      <c r="I55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
@@ -7330,20 +7088,13 @@
         </is>
       </c>
     </row>
+    <row r="59"/>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B60" s="6" t="n"/>
-      <c r="C60" s="6" t="n"/>
-      <c r="D60" s="6" t="n"/>
-      <c r="E60" s="6" t="n"/>
-      <c r="F60" s="6" t="n"/>
-      <c r="G60" s="6" t="n"/>
-      <c r="H60" s="6" t="n"/>
-      <c r="I60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
@@ -7391,6 +7142,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J61" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
@@ -7426,6 +7182,11 @@
       <c r="I62" s="8" t="n">
         <v>15.8</v>
       </c>
+      <c r="J62" s="22" t="inlineStr">
+        <is>
+          <t>Diseña productos, experiencias y servicios turísticos en contextos territoriales y organizacionales, garantizando innovación, sostenibilidad y estándares de calidad internacional.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
@@ -7461,6 +7222,11 @@
       <c r="I63" s="12" t="n">
         <v>47.4</v>
       </c>
+      <c r="J63" s="22" t="inlineStr">
+        <is>
+          <t>Formula estrategias de planificación y comercialización turística en destinos y organizaciones del sector, asegurando competitividad y posicionamiento en el mercado.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
@@ -7496,6 +7262,11 @@
       <c r="I64" s="8" t="n">
         <v>68.40000000000001</v>
       </c>
+      <c r="J64" s="22" t="inlineStr">
+        <is>
+          <t>Optimiza procesos de gestión y operación turística en empresas y emprendimientos del sector, garantizando eficiencia, rentabilidad y mejora continua.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
@@ -7531,6 +7302,11 @@
       <c r="I65" s="12" t="n">
         <v>31.6</v>
       </c>
+      <c r="J65" s="22" t="inlineStr">
+        <is>
+          <t>Evalúa proyectos y servicios turísticos en función del análisis de mercado y segmentación de la demanda, fundamentando decisiones estratégicas sostenibles.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
@@ -7566,6 +7342,11 @@
       <c r="I66" s="8" t="n">
         <v>31.6</v>
       </c>
+      <c r="J66" s="22" t="inlineStr">
+        <is>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
@@ -7601,6 +7382,11 @@
       <c r="I67" s="12" t="n">
         <v>47.4</v>
       </c>
+      <c r="J67" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
@@ -7636,6 +7422,11 @@
       <c r="I68" s="8" t="n">
         <v>68.40000000000001</v>
       </c>
+      <c r="J68" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
@@ -7671,21 +7462,19 @@
       <c r="I69" s="12" t="n">
         <v>15.8</v>
       </c>
-    </row>
+      <c r="J69" s="22" t="inlineStr">
+        <is>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70"/>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B71" s="6" t="n"/>
-      <c r="C71" s="6" t="n"/>
-      <c r="D71" s="6" t="n"/>
-      <c r="E71" s="6" t="n"/>
-      <c r="F71" s="6" t="n"/>
-      <c r="G71" s="6" t="n"/>
-      <c r="H71" s="6" t="n"/>
-      <c r="I71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="7" t="inlineStr">
@@ -7711,20 +7500,14 @@
         </is>
       </c>
     </row>
+    <row r="74"/>
+    <row r="75"/>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B76" s="6" t="n"/>
-      <c r="C76" s="6" t="n"/>
-      <c r="D76" s="6" t="n"/>
-      <c r="E76" s="6" t="n"/>
-      <c r="F76" s="6" t="n"/>
-      <c r="G76" s="6" t="n"/>
-      <c r="H76" s="6" t="n"/>
-      <c r="I76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="7" t="inlineStr">
@@ -7769,12 +7552,6 @@
           <t>CE3 / CT3</t>
         </is>
       </c>
-      <c r="C79" s="16" t="n"/>
-      <c r="D79" s="16" t="n"/>
-      <c r="E79" s="16" t="n"/>
-      <c r="F79" s="16" t="n"/>
-      <c r="G79" s="16" t="n"/>
-      <c r="H79" s="16" t="n"/>
       <c r="I79" s="19" t="n">
         <v>100</v>
       </c>
@@ -7805,12 +7582,6 @@
           <t>CE2 / CT2</t>
         </is>
       </c>
-      <c r="C81" s="16" t="n"/>
-      <c r="D81" s="16" t="n"/>
-      <c r="E81" s="16" t="n"/>
-      <c r="F81" s="16" t="n"/>
-      <c r="G81" s="16" t="n"/>
-      <c r="H81" s="16" t="n"/>
       <c r="I81" s="19" t="n">
         <v>100</v>
       </c>
@@ -7841,12 +7612,6 @@
           <t>CE3 / CT3</t>
         </is>
       </c>
-      <c r="C83" s="16" t="n"/>
-      <c r="D83" s="16" t="n"/>
-      <c r="E83" s="16" t="n"/>
-      <c r="F83" s="16" t="n"/>
-      <c r="G83" s="16" t="n"/>
-      <c r="H83" s="16" t="n"/>
       <c r="I83" s="19" t="n">
         <v>94.7</v>
       </c>
@@ -7877,12 +7642,6 @@
           <t>CE1 / CT4</t>
         </is>
       </c>
-      <c r="C85" s="16" t="n"/>
-      <c r="D85" s="16" t="n"/>
-      <c r="E85" s="16" t="n"/>
-      <c r="F85" s="16" t="n"/>
-      <c r="G85" s="16" t="n"/>
-      <c r="H85" s="16" t="n"/>
       <c r="I85" s="19" t="n">
         <v>94.7</v>
       </c>
@@ -7950,7 +7709,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I108"/>
+  <dimension ref="A1:J108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -7959,6 +7718,7 @@
     <col width="17" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="70" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7975,20 +7735,13 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>══ TA1 — 42 estudiantes ══</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -7996,14 +7749,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
@@ -8117,20 +7862,13 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B10" s="6" t="n"/>
-      <c r="C10" s="6" t="n"/>
-      <c r="D10" s="6" t="n"/>
-      <c r="E10" s="6" t="n"/>
-      <c r="F10" s="6" t="n"/>
-      <c r="G10" s="6" t="n"/>
-      <c r="H10" s="6" t="n"/>
-      <c r="I10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
@@ -8178,6 +7916,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J11" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -8213,6 +7956,11 @@
       <c r="I12" s="8" t="n">
         <v>92.90000000000001</v>
       </c>
+      <c r="J12" s="22" t="inlineStr">
+        <is>
+          <t>Diseña productos turísticos incorporando TIC's, saberes ancestrales, interculturalidad y equidad de género, para generar valor social, económico y cultural.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -8248,6 +7996,11 @@
       <c r="I13" s="12" t="n">
         <v>71.40000000000001</v>
       </c>
+      <c r="J13" s="22" t="inlineStr">
+        <is>
+          <t>Interpreta áreas naturales y patrimoniales mediante principios de educación ambiental y sostenibilidad para promover una participación turística responsable y bio-consciente.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -8283,6 +8036,11 @@
       <c r="I14" s="8" t="n">
         <v>88.09999999999999</v>
       </c>
+      <c r="J14" s="22" t="inlineStr">
+        <is>
+          <t>Aplica herramientas tecnológicas y trabajo multidisciplinario para mejorar la gestión y operación turística sostenible.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -8318,6 +8076,11 @@
       <c r="I15" s="12" t="n">
         <v>92.90000000000001</v>
       </c>
+      <c r="J15" s="22" t="inlineStr">
+        <is>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -8353,6 +8116,11 @@
       <c r="I16" s="8" t="n">
         <v>81</v>
       </c>
+      <c r="J16" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -8388,6 +8156,11 @@
       <c r="I17" s="12" t="n">
         <v>85.7</v>
       </c>
+      <c r="J17" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -8423,21 +8196,19 @@
       <c r="I18" s="8" t="n">
         <v>88.09999999999999</v>
       </c>
-    </row>
+      <c r="J18" s="22" t="inlineStr">
+        <is>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B20" s="6" t="n"/>
-      <c r="C20" s="6" t="n"/>
-      <c r="D20" s="6" t="n"/>
-      <c r="E20" s="6" t="n"/>
-      <c r="F20" s="6" t="n"/>
-      <c r="G20" s="6" t="n"/>
-      <c r="H20" s="6" t="n"/>
-      <c r="I20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
@@ -8463,20 +8234,14 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B25" s="6" t="n"/>
-      <c r="C25" s="6" t="n"/>
-      <c r="D25" s="6" t="n"/>
-      <c r="E25" s="6" t="n"/>
-      <c r="F25" s="6" t="n"/>
-      <c r="G25" s="6" t="n"/>
-      <c r="H25" s="6" t="n"/>
-      <c r="I25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
@@ -8521,12 +8286,6 @@
           <t>CT3</t>
         </is>
       </c>
-      <c r="C28" s="16" t="n"/>
-      <c r="D28" s="16" t="n"/>
-      <c r="E28" s="16" t="n"/>
-      <c r="F28" s="16" t="n"/>
-      <c r="G28" s="16" t="n"/>
-      <c r="H28" s="16" t="n"/>
       <c r="I28" s="19" t="n">
         <v>100</v>
       </c>
@@ -8557,12 +8316,6 @@
           <t>CE1 / CT1</t>
         </is>
       </c>
-      <c r="C30" s="16" t="n"/>
-      <c r="D30" s="16" t="n"/>
-      <c r="E30" s="16" t="n"/>
-      <c r="F30" s="16" t="n"/>
-      <c r="G30" s="16" t="n"/>
-      <c r="H30" s="16" t="n"/>
       <c r="I30" s="19" t="n">
         <v>100</v>
       </c>
@@ -8593,12 +8346,6 @@
           <t>CE2 / CT3</t>
         </is>
       </c>
-      <c r="C32" s="16" t="n"/>
-      <c r="D32" s="16" t="n"/>
-      <c r="E32" s="16" t="n"/>
-      <c r="F32" s="16" t="n"/>
-      <c r="G32" s="16" t="n"/>
-      <c r="H32" s="16" t="n"/>
       <c r="I32" s="19" t="n">
         <v>100</v>
       </c>
@@ -8629,12 +8376,6 @@
           <t>CE3 / CT4</t>
         </is>
       </c>
-      <c r="C34" s="16" t="n"/>
-      <c r="D34" s="16" t="n"/>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="16" t="n"/>
-      <c r="G34" s="16" t="n"/>
-      <c r="H34" s="16" t="n"/>
       <c r="I34" s="19" t="n">
         <v>100</v>
       </c>
@@ -8665,12 +8406,6 @@
           <t>CE1 / CT1</t>
         </is>
       </c>
-      <c r="C36" s="16" t="n"/>
-      <c r="D36" s="16" t="n"/>
-      <c r="E36" s="16" t="n"/>
-      <c r="F36" s="16" t="n"/>
-      <c r="G36" s="16" t="n"/>
-      <c r="H36" s="16" t="n"/>
       <c r="I36" s="19" t="n">
         <v>100</v>
       </c>
@@ -8701,12 +8436,6 @@
           <t>CE3 / CT4</t>
         </is>
       </c>
-      <c r="C38" s="16" t="n"/>
-      <c r="D38" s="16" t="n"/>
-      <c r="E38" s="16" t="n"/>
-      <c r="F38" s="16" t="n"/>
-      <c r="G38" s="16" t="n"/>
-      <c r="H38" s="16" t="n"/>
       <c r="I38" s="19" t="n">
         <v>97.59999999999999</v>
       </c>
@@ -8737,12 +8466,6 @@
           <t>CE2 / CT3</t>
         </is>
       </c>
-      <c r="C40" s="16" t="n"/>
-      <c r="D40" s="16" t="n"/>
-      <c r="E40" s="16" t="n"/>
-      <c r="F40" s="16" t="n"/>
-      <c r="G40" s="16" t="n"/>
-      <c r="H40" s="16" t="n"/>
       <c r="I40" s="19" t="n">
         <v>97.59999999999999</v>
       </c>
@@ -8773,12 +8496,6 @@
           <t>CT2</t>
         </is>
       </c>
-      <c r="C42" s="16" t="n"/>
-      <c r="D42" s="16" t="n"/>
-      <c r="E42" s="16" t="n"/>
-      <c r="F42" s="16" t="n"/>
-      <c r="G42" s="16" t="n"/>
-      <c r="H42" s="16" t="n"/>
       <c r="I42" s="19" t="n">
         <v>97.59999999999999</v>
       </c>
@@ -8809,12 +8526,6 @@
           <t>CT3</t>
         </is>
       </c>
-      <c r="C44" s="16" t="n"/>
-      <c r="D44" s="16" t="n"/>
-      <c r="E44" s="16" t="n"/>
-      <c r="F44" s="16" t="n"/>
-      <c r="G44" s="16" t="n"/>
-      <c r="H44" s="16" t="n"/>
       <c r="I44" s="19" t="n">
         <v>95.2</v>
       </c>
@@ -8845,12 +8556,6 @@
           <t>CT2</t>
         </is>
       </c>
-      <c r="C46" s="16" t="n"/>
-      <c r="D46" s="16" t="n"/>
-      <c r="E46" s="16" t="n"/>
-      <c r="F46" s="16" t="n"/>
-      <c r="G46" s="16" t="n"/>
-      <c r="H46" s="16" t="n"/>
       <c r="I46" s="19" t="n">
         <v>95.2</v>
       </c>
@@ -8881,12 +8586,6 @@
           <t>CT3</t>
         </is>
       </c>
-      <c r="C48" s="16" t="n"/>
-      <c r="D48" s="16" t="n"/>
-      <c r="E48" s="16" t="n"/>
-      <c r="F48" s="16" t="n"/>
-      <c r="G48" s="16" t="n"/>
-      <c r="H48" s="16" t="n"/>
       <c r="I48" s="19" t="n">
         <v>95.2</v>
       </c>
@@ -8917,12 +8616,6 @@
           <t>CT3</t>
         </is>
       </c>
-      <c r="C50" s="16" t="n"/>
-      <c r="D50" s="16" t="n"/>
-      <c r="E50" s="16" t="n"/>
-      <c r="F50" s="16" t="n"/>
-      <c r="G50" s="16" t="n"/>
-      <c r="H50" s="16" t="n"/>
       <c r="I50" s="19" t="n">
         <v>92.90000000000001</v>
       </c>
@@ -8953,12 +8646,6 @@
           <t>CE2 / CT3</t>
         </is>
       </c>
-      <c r="C52" s="16" t="n"/>
-      <c r="D52" s="16" t="n"/>
-      <c r="E52" s="16" t="n"/>
-      <c r="F52" s="16" t="n"/>
-      <c r="G52" s="16" t="n"/>
-      <c r="H52" s="16" t="n"/>
       <c r="I52" s="19" t="n">
         <v>90.5</v>
       </c>
@@ -8978,20 +8665,14 @@
         <v>90.5</v>
       </c>
     </row>
+    <row r="54"/>
+    <row r="55"/>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
           <t>══ TA2 — 95 estudiantes ══</t>
         </is>
       </c>
-      <c r="B56" s="4" t="n"/>
-      <c r="C56" s="4" t="n"/>
-      <c r="D56" s="4" t="n"/>
-      <c r="E56" s="4" t="n"/>
-      <c r="F56" s="4" t="n"/>
-      <c r="G56" s="4" t="n"/>
-      <c r="H56" s="4" t="n"/>
-      <c r="I56" s="4" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
@@ -8999,14 +8680,6 @@
           <t>Resultado global de cohorte</t>
         </is>
       </c>
-      <c r="B57" s="6" t="n"/>
-      <c r="C57" s="6" t="n"/>
-      <c r="D57" s="6" t="n"/>
-      <c r="E57" s="6" t="n"/>
-      <c r="F57" s="6" t="n"/>
-      <c r="G57" s="6" t="n"/>
-      <c r="H57" s="6" t="n"/>
-      <c r="I57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
@@ -9120,20 +8793,13 @@
         </is>
       </c>
     </row>
+    <row r="61"/>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
           <t>Logro y distribución por competencia</t>
         </is>
       </c>
-      <c r="B62" s="6" t="n"/>
-      <c r="C62" s="6" t="n"/>
-      <c r="D62" s="6" t="n"/>
-      <c r="E62" s="6" t="n"/>
-      <c r="F62" s="6" t="n"/>
-      <c r="G62" s="6" t="n"/>
-      <c r="H62" s="6" t="n"/>
-      <c r="I62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
@@ -9181,6 +8847,11 @@
           <t>% Sobres.</t>
         </is>
       </c>
+      <c r="J63" s="21" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
@@ -9216,6 +8887,11 @@
       <c r="I64" s="8" t="n">
         <v>86.3</v>
       </c>
+      <c r="J64" s="22" t="inlineStr">
+        <is>
+          <t>Diseña productos turísticos incorporando TIC's, saberes ancestrales, interculturalidad y equidad de género, para generar valor social, económico y cultural.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
@@ -9251,6 +8927,11 @@
       <c r="I65" s="12" t="n">
         <v>92.59999999999999</v>
       </c>
+      <c r="J65" s="22" t="inlineStr">
+        <is>
+          <t>Interpreta áreas naturales y patrimoniales mediante principios de educación ambiental y sostenibilidad para promover una participación turística responsable y bio-consciente.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
@@ -9286,6 +8967,11 @@
       <c r="I66" s="8" t="n">
         <v>90.5</v>
       </c>
+      <c r="J66" s="22" t="inlineStr">
+        <is>
+          <t>Aplica herramientas tecnológicas y trabajo multidisciplinario para mejorar la gestión y operación turística sostenible.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
@@ -9321,6 +9007,11 @@
       <c r="I67" s="12" t="n">
         <v>91.59999999999999</v>
       </c>
+      <c r="J67" s="22" t="inlineStr">
+        <is>
+          <t>Formula proyectos turísticos innovadores para implementar iniciativas alineadas a políticas públicas y tendencias globales.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
@@ -9356,6 +9047,11 @@
       <c r="I68" s="8" t="n">
         <v>90.5</v>
       </c>
+      <c r="J68" s="22" t="inlineStr">
+        <is>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="11" t="inlineStr">
@@ -9391,6 +9087,11 @@
       <c r="I69" s="12" t="n">
         <v>74.7</v>
       </c>
+      <c r="J69" s="22" t="inlineStr">
+        <is>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
@@ -9426,6 +9127,11 @@
       <c r="I70" s="8" t="n">
         <v>92.59999999999999</v>
       </c>
+      <c r="J70" s="22" t="inlineStr">
+        <is>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="11" t="inlineStr">
@@ -9461,21 +9167,19 @@
       <c r="I71" s="12" t="n">
         <v>90.5</v>
       </c>
-    </row>
+      <c r="J71" s="22" t="inlineStr">
+        <is>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72"/>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
           <t>Ítems críticos (&lt;50% de aciertos, nivel Insuficiente)</t>
         </is>
       </c>
-      <c r="B73" s="6" t="n"/>
-      <c r="C73" s="6" t="n"/>
-      <c r="D73" s="6" t="n"/>
-      <c r="E73" s="6" t="n"/>
-      <c r="F73" s="6" t="n"/>
-      <c r="G73" s="6" t="n"/>
-      <c r="H73" s="6" t="n"/>
-      <c r="I73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="7" t="inlineStr">
@@ -9501,20 +9205,14 @@
         </is>
       </c>
     </row>
+    <row r="76"/>
+    <row r="77"/>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>
           <t>Ítems sobresalientes (≥90% de aciertos, nivel Sobresaliente)</t>
         </is>
       </c>
-      <c r="B78" s="6" t="n"/>
-      <c r="C78" s="6" t="n"/>
-      <c r="D78" s="6" t="n"/>
-      <c r="E78" s="6" t="n"/>
-      <c r="F78" s="6" t="n"/>
-      <c r="G78" s="6" t="n"/>
-      <c r="H78" s="6" t="n"/>
-      <c r="I78" s="6" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="7" t="inlineStr">
@@ -9559,12 +9257,6 @@
           <t>CT3</t>
         </is>
       </c>
-      <c r="C81" s="16" t="n"/>
-      <c r="D81" s="16" t="n"/>
-      <c r="E81" s="16" t="n"/>
-      <c r="F81" s="16" t="n"/>
-      <c r="G81" s="16" t="n"/>
-      <c r="H81" s="16" t="n"/>
       <c r="I81" s="19" t="n">
         <v>100</v>
       </c>
@@ -9595,12 +9287,6 @@
           <t>CT3</t>
         </is>
       </c>
-      <c r="C83" s="16" t="n"/>
-      <c r="D83" s="16" t="n"/>
-      <c r="E83" s="16" t="n"/>
-      <c r="F83" s="16" t="n"/>
-      <c r="G83" s="16" t="n"/>
-      <c r="H83" s="16" t="n"/>
       <c r="I83" s="19" t="n">
         <v>98.90000000000001</v>
       </c>
@@ -9631,12 +9317,6 @@
           <t>CE3 / CT4</t>
         </is>
       </c>
-      <c r="C85" s="16" t="n"/>
-      <c r="D85" s="16" t="n"/>
-      <c r="E85" s="16" t="n"/>
-      <c r="F85" s="16" t="n"/>
-      <c r="G85" s="16" t="n"/>
-      <c r="H85" s="16" t="n"/>
       <c r="I85" s="19" t="n">
         <v>98.90000000000001</v>
       </c>
@@ -9667,12 +9347,6 @@
           <t>CT3</t>
         </is>
       </c>
-      <c r="C87" s="16" t="n"/>
-      <c r="D87" s="16" t="n"/>
-      <c r="E87" s="16" t="n"/>
-      <c r="F87" s="16" t="n"/>
-      <c r="G87" s="16" t="n"/>
-      <c r="H87" s="16" t="n"/>
       <c r="I87" s="19" t="n">
         <v>98.90000000000001</v>
       </c>
@@ -9703,12 +9377,6 @@
           <t>CE1 / CE4</t>
         </is>
       </c>
-      <c r="C89" s="16" t="n"/>
-      <c r="D89" s="16" t="n"/>
-      <c r="E89" s="16" t="n"/>
-      <c r="F89" s="16" t="n"/>
-      <c r="G89" s="16" t="n"/>
-      <c r="H89" s="16" t="n"/>
       <c r="I89" s="19" t="n">
         <v>98.90000000000001</v>
       </c>
@@ -9739,12 +9407,6 @@
           <t>CE1 / CE4</t>
         </is>
       </c>
-      <c r="C91" s="16" t="n"/>
-      <c r="D91" s="16" t="n"/>
-      <c r="E91" s="16" t="n"/>
-      <c r="F91" s="16" t="n"/>
-      <c r="G91" s="16" t="n"/>
-      <c r="H91" s="16" t="n"/>
       <c r="I91" s="19" t="n">
         <v>97.90000000000001</v>
       </c>
@@ -9775,12 +9437,6 @@
           <t>CE2 / CT3</t>
         </is>
       </c>
-      <c r="C93" s="16" t="n"/>
-      <c r="D93" s="16" t="n"/>
-      <c r="E93" s="16" t="n"/>
-      <c r="F93" s="16" t="n"/>
-      <c r="G93" s="16" t="n"/>
-      <c r="H93" s="16" t="n"/>
       <c r="I93" s="19" t="n">
         <v>97.90000000000001</v>
       </c>
@@ -9811,12 +9467,6 @@
           <t>CE4 / CT2</t>
         </is>
       </c>
-      <c r="C95" s="16" t="n"/>
-      <c r="D95" s="16" t="n"/>
-      <c r="E95" s="16" t="n"/>
-      <c r="F95" s="16" t="n"/>
-      <c r="G95" s="16" t="n"/>
-      <c r="H95" s="16" t="n"/>
       <c r="I95" s="19" t="n">
         <v>97.90000000000001</v>
       </c>
@@ -9847,12 +9497,6 @@
           <t>CE1 / CT1</t>
         </is>
       </c>
-      <c r="C97" s="16" t="n"/>
-      <c r="D97" s="16" t="n"/>
-      <c r="E97" s="16" t="n"/>
-      <c r="F97" s="16" t="n"/>
-      <c r="G97" s="16" t="n"/>
-      <c r="H97" s="16" t="n"/>
       <c r="I97" s="19" t="n">
         <v>96.8</v>
       </c>
@@ -9883,12 +9527,6 @@
           <t>CE1 / CT1</t>
         </is>
       </c>
-      <c r="C99" s="16" t="n"/>
-      <c r="D99" s="16" t="n"/>
-      <c r="E99" s="16" t="n"/>
-      <c r="F99" s="16" t="n"/>
-      <c r="G99" s="16" t="n"/>
-      <c r="H99" s="16" t="n"/>
       <c r="I99" s="19" t="n">
         <v>96.8</v>
       </c>
@@ -9919,12 +9557,6 @@
           <t>CE3 / CT4</t>
         </is>
       </c>
-      <c r="C101" s="16" t="n"/>
-      <c r="D101" s="16" t="n"/>
-      <c r="E101" s="16" t="n"/>
-      <c r="F101" s="16" t="n"/>
-      <c r="G101" s="16" t="n"/>
-      <c r="H101" s="16" t="n"/>
       <c r="I101" s="19" t="n">
         <v>96.8</v>
       </c>
@@ -9955,12 +9587,6 @@
           <t>CE3 / CT4</t>
         </is>
       </c>
-      <c r="C103" s="16" t="n"/>
-      <c r="D103" s="16" t="n"/>
-      <c r="E103" s="16" t="n"/>
-      <c r="F103" s="16" t="n"/>
-      <c r="G103" s="16" t="n"/>
-      <c r="H103" s="16" t="n"/>
       <c r="I103" s="19" t="n">
         <v>96.8</v>
       </c>
@@ -9991,12 +9617,6 @@
           <t>CE4 / CT2</t>
         </is>
       </c>
-      <c r="C105" s="16" t="n"/>
-      <c r="D105" s="16" t="n"/>
-      <c r="E105" s="16" t="n"/>
-      <c r="F105" s="16" t="n"/>
-      <c r="G105" s="16" t="n"/>
-      <c r="H105" s="16" t="n"/>
       <c r="I105" s="19" t="n">
         <v>96.8</v>
       </c>
@@ -10027,12 +9647,6 @@
           <t>CE4 / CT2</t>
         </is>
       </c>
-      <c r="C107" s="16" t="n"/>
-      <c r="D107" s="16" t="n"/>
-      <c r="E107" s="16" t="n"/>
-      <c r="F107" s="16" t="n"/>
-      <c r="G107" s="16" t="n"/>
-      <c r="H107" s="16" t="n"/>
       <c r="I107" s="19" t="n">
         <v>95.8</v>
       </c>

</xml_diff>

<commit_message>
Agrega filtro por tipo de competencia y corrige descripciones de Contabilidad
Al hacer clic en Especificas (CE) o Transversales (CT) en la carrera,
recalcula Distribucion de niveles y filtra/atenua Logro por competencia,
mapa de calor y Resultados por item. Diferencia CE/CT con dos colores
(azul/naranja) en los graficos de competencia, reordena las tarjetas KPI
por ronda (TA1 completo, luego TA2) y actualiza las descripciones de
Contabilidad y Auditoria desde el cuadro oficial corregido.
</commit_message>
<xml_diff>
--- a/data/Cuadros_oficiales_por_carrera.xlsx
+++ b/data/Cuadros_oficiales_por_carrera.xlsx
@@ -549,7 +549,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -676,7 +675,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -1056,7 +1054,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
@@ -1141,8 +1138,6 @@
         <v>46.7</v>
       </c>
     </row>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
@@ -1212,8 +1207,6 @@
         <v>91.2</v>
       </c>
     </row>
-    <row r="34"/>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
@@ -1340,7 +1333,6 @@
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
@@ -1720,7 +1712,6 @@
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
@@ -1775,8 +1766,6 @@
         <v>31.7</v>
       </c>
     </row>
-    <row r="57"/>
-    <row r="58"/>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
@@ -2386,7 +2375,7 @@
       </c>
       <c r="J15" s="22" t="inlineStr">
         <is>
-          <t>Analiza situaciones profesionales y toma decisiones fundamentadas considerando impactos sociales, ambientales, económicos y tecnológicos, actuando con responsabilidad, integridad y compromiso con el desarrollo sostenible en contextos locales y globales.</t>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
         </is>
       </c>
     </row>
@@ -2426,7 +2415,7 @@
       </c>
       <c r="J16" s="22" t="inlineStr">
         <is>
-          <t>Comunica ideas con claridad y sustento técnico, y colabora eficazmente en equipos diversos e interdisciplinarios, contribuyendo activamente a la construcción de soluciones en entornos profesionales, multiculturales y digitales.</t>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2455,7 @@
       </c>
       <c r="J17" s="22" t="inlineStr">
         <is>
-          <t>Gestiona información y conocimiento con rigor metodológico, actualizándose de manera autónoma y aplicando nuevos saberes para resolver problemas complejos en contextos dinámicos y cambiantes.</t>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
         </is>
       </c>
     </row>
@@ -2506,7 +2495,7 @@
       </c>
       <c r="J18" s="22" t="inlineStr">
         <is>
-          <t>Integra tecnologías digitales, análisis de datos y herramientas emergentes de manera crítica, ética y estratégica para generar soluciones pertinentes y sostenibles en contextos profesionales y sociales.</t>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
         </is>
       </c>
     </row>
@@ -3020,7 +3009,7 @@
       </c>
       <c r="J45" s="22" t="inlineStr">
         <is>
-          <t>Analiza situaciones profesionales y toma decisiones fundamentadas considerando impactos sociales, ambientales, económicos y tecnológicos, actuando con responsabilidad, integridad y compromiso con el desarrollo sostenible en contextos locales y globales.</t>
+          <t>Analiza problemas del contexto profesional y social, a partir de información pertinente, para proponer soluciones fundamentadas, viables y contextualizadas.</t>
         </is>
       </c>
     </row>
@@ -3060,7 +3049,7 @@
       </c>
       <c r="J46" s="22" t="inlineStr">
         <is>
-          <t>Comunica ideas con claridad y sustento técnico, y colabora eficazmente en equipos diversos e interdisciplinarios, contribuyendo activamente a la construcción de soluciones en entornos profesionales, multiculturales y digitales.</t>
+          <t>Comunica ideas, argumentos y resultados de manera clara, estructurada y pertinente, para facilitar la comprensión, la colaboración y la toma de decisiones.</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3089,7 @@
       </c>
       <c r="J47" s="22" t="inlineStr">
         <is>
-          <t>Gestiona información y conocimiento con rigor metodológico, actualizándose de manera autónoma y aplicando nuevos saberes para resolver problemas complejos en contextos dinámicos y cambiantes.</t>
+          <t>Gestiona su aprendizaje de manera autónoma para actualizar sus conocimientos y adaptar su desempeño a los cambios del entorno.</t>
         </is>
       </c>
     </row>
@@ -3140,7 +3129,7 @@
       </c>
       <c r="J48" s="22" t="inlineStr">
         <is>
-          <t>Integra tecnologías digitales, análisis de datos y herramientas emergentes de manera crítica, ética y estratégica para generar soluciones pertinentes y sostenibles en contextos profesionales y sociales.</t>
+          <t>Utiliza tecnologías, datos y entornos digitales de manera crítica, segura y pertinente para gestionar información, interactuar responsablemente y generar soluciones de valor.</t>
         </is>
       </c>
     </row>
@@ -3433,7 +3422,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -3560,7 +3548,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -3900,7 +3887,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
@@ -4045,8 +4031,6 @@
         <v>47.5</v>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
@@ -4116,8 +4100,6 @@
         <v>90</v>
       </c>
     </row>
-    <row r="37"/>
-    <row r="38"/>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
@@ -4244,7 +4226,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="5" t="inlineStr">
         <is>
@@ -4584,7 +4565,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
@@ -4654,8 +4634,6 @@
         <v>21.9</v>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
@@ -4767,7 +4745,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -4894,7 +4871,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -5114,7 +5090,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
@@ -5146,8 +5121,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
@@ -5292,8 +5265,6 @@
         <v>90.3</v>
       </c>
     </row>
-    <row r="32"/>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
@@ -5420,7 +5391,6 @@
         </is>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
@@ -5640,7 +5610,6 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
@@ -5672,8 +5641,6 @@
         </is>
       </c>
     </row>
-    <row r="50"/>
-    <row r="51"/>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
@@ -6035,7 +6002,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -6162,7 +6128,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -6542,7 +6507,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
@@ -6574,8 +6538,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
@@ -6960,8 +6922,6 @@
         <v>100</v>
       </c>
     </row>
-    <row r="52"/>
-    <row r="53"/>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
@@ -7088,7 +7048,6 @@
         </is>
       </c>
     </row>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
@@ -7468,7 +7427,6 @@
         </is>
       </c>
     </row>
-    <row r="70"/>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
@@ -7500,8 +7458,6 @@
         </is>
       </c>
     </row>
-    <row r="74"/>
-    <row r="75"/>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
@@ -7735,7 +7691,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -7862,7 +7817,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
@@ -8202,7 +8156,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
@@ -8234,8 +8187,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
-    <row r="24"/>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
@@ -8665,8 +8616,6 @@
         <v>90.5</v>
       </c>
     </row>
-    <row r="54"/>
-    <row r="55"/>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
@@ -8793,7 +8742,6 @@
         </is>
       </c>
     </row>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
@@ -9173,7 +9121,6 @@
         </is>
       </c>
     </row>
-    <row r="72"/>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
@@ -9205,8 +9152,6 @@
         </is>
       </c>
     </row>
-    <row r="76"/>
-    <row r="77"/>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
         <is>

</xml_diff>